<commit_message>
feat: add clickable row jump buttons in transactions sheet
</commit_message>
<xml_diff>
--- a/personal_expense_tracking_template.xlsx
+++ b/personal_expense_tracking_template.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,8 +40,11 @@
       <b val="1"/>
       <sz val="14"/>
     </font>
+    <font>
+      <color rgb="001F4E78"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -53,8 +56,23 @@
         <fgColor rgb="004F81BD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F75B5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -62,11 +80,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B4C6E7"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B4C6E7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B4C6E7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B4C6E7"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -74,6 +106,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1000"/>
+  <dimension ref="A1:K1000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -450,6 +491,8 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -493,6 +536,11 @@
           <t>Year</t>
         </is>
       </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Quick Add Rows</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="F2">
@@ -507,6 +555,15 @@
         <f>IF(A2="","",YEAR(A2))</f>
         <v/>
       </c>
+      <c r="J2" s="6">
+        <f>HYPERLINK("#A"&amp;IFERROR(MATCH(TRUE,INDEX($A$2:$A$1000="",0),0)+1,1001),"Add 1 Row")</f>
+        <v/>
+      </c>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>Jump to next input row</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="F3">
@@ -520,6 +577,15 @@
       <c r="H3">
         <f>IF(A3="","",YEAR(A3))</f>
         <v/>
+      </c>
+      <c r="J3" s="6">
+        <f>HYPERLINK("#A"&amp;MIN(1001,IFERROR(MATCH(TRUE,INDEX($A$2:$A$1000="",0),0)+10,1001)),"Add 10 Rows")</f>
+        <v/>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>Jump 10 rows below next input row</t>
+        </is>
       </c>
     </row>
     <row r="4">

</xml_diff>